<commit_message>
Ground protocol architecture decisions
</commit_message>
<xml_diff>
--- a/docs/planning/sheets/jarvis_roadmap.xlsx
+++ b/docs/planning/sheets/jarvis_roadmap.xlsx
@@ -805,7 +805,7 @@
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Near-term priority: prove one v0 protocol loop end to end: protocol lock, schemas, version and capability negotiation, adapter contract, Garden POC mapping, portable export, and conformance fixtures. Garden POC is the product proof before main Garden adopts the protocol. Keep scope narrow: protocol records first, Garden POC plus one CLI/existing-agent wrapper, evidence and learning captured during work.</t>
+          <t>Near-term priority: prove one v0 protocol loop end to end: protocol lock, schemas, version and capability negotiation, adapter contract, Garden POC mapping, portable export, and conformance fixtures. Garden POC is the product proof before main Garden adopts the protocol. Keep scope narrow: protocol records first, Garden POC plus one real existing-agent adapter, evidence and learning captured during work.</t>
         </is>
       </c>
       <c r="B4" s="30" t="n"/>
@@ -927,14 +927,14 @@
       <c r="G7" s="22" t="inlineStr">
         <is>
           <t>- choose Garden POC as the first product proof
-- choose one CLI/external-agent wrapper
+- choose one real existing-agent adapter
 - define Garden-private fields that stay out of export
 - define demo success path</t>
         </is>
       </c>
       <c r="H7" s="23" t="inlineStr">
         <is>
-          <t>Protocol lock is the source for schema work, Garden POC and wrapper targets are named, and no new runtime/product assumptions enter Jarvis.</t>
+          <t>Protocol lock is the source for schema work, Garden POC and adapter targets are named, and no new runtime/product assumptions enter Jarvis.</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       <c r="F8" s="25" t="inlineStr">
         <is>
           <t>- draft adapter contract
-- define AgentWorker wrapper surface
+- define AgentWorker adapter surface
 - define tool/action to PolicyDecision mapping
 - define limitations field for unsupported concepts</t>
         </is>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="F9" s="21" t="inlineStr">
         <is>
-          <t>- create CLI/existing-agent wrapper plan
+          <t>- create CLI/existing-agent adapter plan
 - capture messages/actions as JarvisEvents
 - capture tool use as PolicyDecision and Evidence
 - capture human correction as Review</t>
@@ -1059,7 +1059,7 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>Prove Jarvis with Garden POC and one existing-agent wrapper.</t>
+          <t>Prove Jarvis with Garden POC and one existing-agent adapter.</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr">
@@ -1073,14 +1073,14 @@
       <c r="E10" s="25" t="inlineStr">
         <is>
           <t>- run schemas against host export
-- run schemas against CLI/wrapper export
+- run schemas against CLI/adapter export
 - compare both exports for same core semantics
 - record gaps as conformance issues</t>
         </is>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>- implement wrapper proof path
+          <t>- implement proof adapter path
 - HumanWorker objective -&gt; AgentWorker action
 - blocked action -&gt; Request
 - human response -&gt; Review or Takeover</t>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="H10" s="25" t="inlineStr">
         <is>
-          <t>Two different host shapes produce valid Jarvis records for the same collaboration loop without sharing runtime, UI, storage, or execution stack.</t>
+          <t>Two different host or adapter shapes produce valid Jarvis records for the same collaboration loop without sharing runtime, UI, storage, or execution stack.</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       <c r="F11" s="21" t="inlineStr">
         <is>
           <t>- write adapter guide
-- document CLI/existing-agent wrapper
+- document CLI/existing-agent adapter
 - document host implementation guide
 - identify next two adapter targets</t>
         </is>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="H11" s="23" t="inlineStr">
         <is>
-          <t>Jarvis has a v0.1 alpha package of protocol docs, schemas, examples, conformance fixtures, Garden POC proof, and one existing-agent wrapper proof.</t>
+          <t>Jarvis has a v0.1 alpha package of protocol docs, schemas, examples, conformance fixtures, Garden POC proof, and one existing-agent adapter proof.</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>- more agent wrappers
+          <t>- more agent adapters
 - MCP/A2A/AG-UI integration notes
 - SDK-neutral adapter examples
 - compatibility badges</t>

</xml_diff>

<commit_message>
Tighten direct protocol wording
</commit_message>
<xml_diff>
--- a/docs/planning/sheets/jarvis_roadmap.xlsx
+++ b/docs/planning/sheets/jarvis_roadmap.xlsx
@@ -781,7 +781,7 @@
     <row r="2" ht="50" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Jarvis is the human-agent collaboration and learning-loop protocol. It defines WorkSession, Policy, Request, Review, Takeover, Contribution, EvidenceManifest, LearningRecord, MemoryProposal, and SkillProposal so existing agents and host products can collaborate with humans without replacing their runtimes.</t>
+          <t>Jarvis is the human-agent collaboration and learning-loop protocol. It defines WorkSession, Policy, Request, Review, Takeover, Contribution, EvidenceManifest, LearningRecord, MemoryProposal, and SkillProposal so existing agents and host products collaborate with humans without replacing their runtimes.</t>
         </is>
       </c>
       <c r="B2" s="32" t="n"/>
@@ -988,7 +988,7 @@
       </c>
       <c r="H8" s="25" t="inlineStr">
         <is>
-          <t>A developer can read the schemas and know exactly how to create a valid WorkSession, Request, Review, Contribution, EvidenceManifest, and LearningRecord.</t>
+          <t>A developer reads the schemas and knows exactly how to create a valid WorkSession, Request, Review, Contribution, EvidenceManifest, and LearningRecord.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adopt OpenAPI communication contract strategy
</commit_message>
<xml_diff>
--- a/docs/planning/sheets/jarvis_roadmap.xlsx
+++ b/docs/planning/sheets/jarvis_roadmap.xlsx
@@ -805,7 +805,7 @@
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Near-term priority: prove one v0 protocol loop end to end: protocol lock, schemas, version and capability negotiation, adapter contract, Garden POC mapping, portable export, and conformance fixtures. Garden POC is the product proof before main Garden adopts the protocol. Keep scope narrow: protocol records first, Garden POC plus one real existing-agent adapter, evidence and learning captured during work.</t>
+          <t>Near-term priority: make Jarvis OpenAPI-ready: protocol lock, OpenAPI 3.1 communication binding, version and capability negotiation, zero-trust security model, portable export, and conformance entry fixtures. Product proof waits behind the protocol contract. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, adapters fourth, product proof last.</t>
         </is>
       </c>
       <c r="B4" s="30" t="n"/>
@@ -831,13 +831,13 @@
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>Schemas + Adapters</t>
+          <t>OpenAPI + Conformance</t>
         </is>
       </c>
       <c r="F5" s="31" t="n"/>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>Proof + Review</t>
+          <t>Proof Readiness</t>
         </is>
       </c>
       <c r="H5" s="31" t="n"/>
@@ -865,7 +865,7 @@
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>Schemas + conformance</t>
+          <t>OpenAPI + conformance</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>Garden POC + demo</t>
+          <t>Product proof</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
@@ -910,31 +910,29 @@
       </c>
       <c r="E7" s="21" t="inlineStr">
         <is>
-          <t>- define schema entry gate
-- list open schema questions
+          <t>- define OpenAPI entry gate
+- list open OpenAPI questions
 - identify version, capability, extension, and error-model gaps
-- prepare schema folder layout</t>
+- prepare OpenAPI component and path layout
+- define zero-trust headers and security schemes</t>
         </is>
       </c>
       <c r="F7" s="21" t="inlineStr">
         <is>
-          <t>- name first adapter targets
-- define what an existing agent must expose
-- map agent steps to JarvisEvent
-- map blocked action to Request</t>
+          <t>- defer adapter implementation
+- name adapter questions only
+- preserve runtime independence</t>
         </is>
       </c>
       <c r="G7" s="22" t="inlineStr">
         <is>
-          <t>- choose Garden POC as the first product proof
-- choose one real existing-agent adapter
-- define Garden-private fields that stay out of export
-- define demo success path</t>
+          <t>- keep Garden POC out of active scope
+- define product-proof prerequisites only</t>
         </is>
       </c>
       <c r="H7" s="23" t="inlineStr">
         <is>
-          <t>Protocol lock is the source for schema work, Garden POC and adapter targets are named, and no new runtime/product assumptions enter Jarvis.</t>
+          <t>Protocol lock is the source for OpenAPI work, OpenAPI 3.1 is the machine-readable communication contract, and no product proof enters this week.</t>
         </is>
       </c>
     </row>
@@ -951,7 +949,7 @@
       </c>
       <c r="C8" s="25" t="inlineStr">
         <is>
-          <t>Create the v0 machine-readable contract.</t>
+          <t>Create the v0 OpenAPI communication contract.</t>
         </is>
       </c>
       <c r="D8" s="25" t="inlineStr">
@@ -964,15 +962,16 @@
       </c>
       <c r="E8" s="25" t="inlineStr">
         <is>
-          <t>- create JSON schemas for core objects
-- create JarvisEvent envelope schema
-- create portable export schema
-- define protocol error codes</t>
+          <t>- create OpenAPI 3.1 document skeleton
+- create components.schemas for core objects
+- create path layout for core operations
+- define protocol error responses
+- define required security headers</t>
         </is>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>- draft adapter contract
+          <t>- document adapter contract questions
 - define AgentWorker adapter surface
 - define tool/action to PolicyDecision mapping
 - define limitations field for unsupported concepts</t>
@@ -980,15 +979,13 @@
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>- create Garden POC mapping table
-- define Garden WorkSession flow
-- define Request inbox behavior
-- define Review and Takeover capture points</t>
+          <t>- keep Garden POC out of active scope
+- define product-proof gate conditions only</t>
         </is>
       </c>
       <c r="H8" s="25" t="inlineStr">
         <is>
-          <t>A developer reads the schemas and knows exactly how to create a valid WorkSession, Request, Review, Contribution, EvidenceManifest, and LearningRecord.</t>
+          <t>A developer reads the OpenAPI contract and knows exactly how to create a valid WorkSession, Request, Review, Contribution, EvidenceManifest, and LearningRecord.</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1018,7 @@
           <t>- build golden-path fixtures
 - build failing fixtures
 - validate status transitions
-- validate export does not require Garden-private fields</t>
+- validate export does not require product-private fields</t>
         </is>
       </c>
       <c r="F9" s="21" t="inlineStr">
@@ -1034,9 +1031,9 @@
       </c>
       <c r="G9" s="22" t="inlineStr">
         <is>
-          <t>- run Garden POC mapping against schemas
-- generate sample WorkSession export
-- show evidence and learning records
+          <t>- keep product proof out of active scope
+- record product-proof prerequisites from conformance only
+- generate protocol-only sample WorkSession export
 - document host-only assumptions separately</t>
         </is>
       </c>
@@ -1059,7 +1056,7 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>Prove Jarvis with Garden POC and one existing-agent adapter.</t>
+          <t>Prove Jarvis with conformance fixtures and one adapter contract.</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr">
@@ -1072,8 +1069,8 @@
       </c>
       <c r="E10" s="25" t="inlineStr">
         <is>
-          <t>- run schemas against host export
-- run schemas against CLI/adapter export
+          <t>- run OpenAPI examples against host export
+- run OpenAPI examples against CLI/adapter export
 - compare both exports for same core semantics
 - record gaps as conformance issues</t>
         </is>
@@ -1088,10 +1085,8 @@
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>- demonstrate Garden POC flow
-- export EvidenceManifest
-- export LearningRecord
-- show human, agent, and pair learning
+          <t>- prepare Garden POC as later product proof
+- define product-private fields that stay out of export
 - update simulation narrative if needed</t>
         </is>
       </c>
@@ -1114,7 +1109,7 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Freeze v0.1 alpha and prepare team/public review.</t>
+          <t>Freeze v0.1 alpha and prepare product-proof review.</t>
         </is>
       </c>
       <c r="D11" s="20" t="inlineStr">
@@ -1127,7 +1122,7 @@
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>- freeze v0.1 schema draft
+          <t>- freeze v0.1 OpenAPI contract
 - publish conformance checklist
 - publish valid/invalid examples
 - define migration policy draft</t>
@@ -1143,15 +1138,15 @@
       </c>
       <c r="G11" s="22" t="inlineStr">
         <is>
-          <t>- publish final demo URL
-- package Garden POC evidence
+          <t>- publish protocol proof walkthrough URL
+- package product-proof readiness notes
 - prepare team walkthrough
 - collect review notes into next-cycle issues</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr">
         <is>
-          <t>Jarvis has a v0.1 alpha package of protocol docs, schemas, examples, conformance fixtures, Garden POC proof, and one existing-agent adapter proof.</t>
+          <t>Jarvis has a v0.1 alpha package of protocol docs, OpenAPI contract, examples, conformance fixtures, product-proof readiness, and one existing-agent adapter contract.</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1163,7 @@
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>Expand only from conformance and proof-host evidence.</t>
+          <t>Expand only from conformance results and product-proof evidence.</t>
         </is>
       </c>
       <c r="D12" s="25" t="inlineStr">
@@ -1198,14 +1193,14 @@
       <c r="G12" s="25" t="inlineStr">
         <is>
           <t>- additional product proofs
-- public demo refresh
+- public proof refresh
 - team onboarding sheet
 - protocol review sessions</t>
         </is>
       </c>
       <c r="H12" s="25" t="inlineStr">
         <is>
-          <t>Expansion is justified by valid exports, conformance failures, adapter pain, and Garden POC evidence, not by adding features from vibes.</t>
+          <t>Expansion is justified by valid exports, conformance failures, adapter pain, and product-proof evidence, not by unproven feature expansion.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harden Jarvis protocol boundary
</commit_message>
<xml_diff>
--- a/docs/planning/sheets/jarvis_roadmap.xlsx
+++ b/docs/planning/sheets/jarvis_roadmap.xlsx
@@ -805,7 +805,7 @@
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Near-term priority: make Jarvis OpenAPI-ready: protocol lock, OpenAPI 3.1 communication binding, version and capability negotiation, zero-trust security model, portable export, and conformance entry fixtures. Product proof waits behind the protocol contract. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, adapters fourth, product proof last.</t>
+          <t>Near-term priority: make Jarvis OpenAPI-ready: protocol lock, OpenAPI 3.1 communication binding, version and capability negotiation, zero-trust security model, portable export, and conformance entry fixtures. Product proof starts only after the protocol contract. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, adapters fourth, product proof last.</t>
         </is>
       </c>
       <c r="B4" s="30" t="n"/>
@@ -949,7 +949,7 @@
       </c>
       <c r="C8" s="25" t="inlineStr">
         <is>
-          <t>Create the v0 OpenAPI communication contract.</t>
+          <t>Create the v0.1 OpenAPI communication contract.</t>
         </is>
       </c>
       <c r="D8" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Address protocol boundary review findings
</commit_message>
<xml_diff>
--- a/docs/planning/sheets/jarvis_roadmap.xlsx
+++ b/docs/planning/sheets/jarvis_roadmap.xlsx
@@ -805,7 +805,7 @@
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Near-term priority: make Jarvis OpenAPI-ready: protocol lock, OpenAPI 3.1 communication binding, version and capability negotiation, zero-trust security model, portable export, and conformance entry fixtures. Product proof starts only after the protocol contract. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, adapters fourth, product proof last.</t>
+          <t>Near-term priority: make Jarvis OpenAPI-ready: protocol lock, OpenAPI 3.1 communication binding, version and capability negotiation, zero-trust security model, portable export, and conformance entry fixtures. Product proof starts only after the protocol contract and conformance entry rules are stable. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, adapters fourth, product proof last.</t>
         </is>
       </c>
       <c r="B4" s="30" t="n"/>
@@ -902,7 +902,7 @@
       </c>
       <c r="D7" s="20" t="inlineStr">
         <is>
-          <t>- freeze v0 protocol lock
+          <t>- freeze v0.1 protocol lock
 - align README, principles, architecture, roadmap
 - keep language direct and host-generic
 - confirm object names and lifecycle</t>

</xml_diff>

<commit_message>
Close Week 2 and set Week 3 focus
</commit_message>
<xml_diff>
--- a/docs/planning/sheets/jarvis_roadmap.xlsx
+++ b/docs/planning/sheets/jarvis_roadmap.xlsx
@@ -781,7 +781,7 @@
     <row r="2" ht="50" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Jarvis is the human-agent collaboration and learning-loop protocol. It defines WorkSession, Policy, Request, Review, Takeover, Contribution, EvidenceManifest, LearningRecord, MemoryProposal, and SkillProposal so existing agents and host products collaborate with humans without replacing their runtimes.</t>
+          <t>Jarvis is the human-agent collaboration and learning-loop protocol. It defines WorkSession, Policy, Request, Review, Takeover, Contribution, EvidenceManifest, LearningRecord, MemoryProposal, and SkillProposal so existing agents and host applications collaborate with humans without replacing their runtimes.</t>
         </is>
       </c>
       <c r="B2" s="32" t="n"/>
@@ -805,7 +805,7 @@
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Near-term priority: make Jarvis OpenAPI-ready: protocol lock, OpenAPI 3.1 communication binding, version and capability negotiation, zero-trust security model, portable export, and conformance entry fixtures. Product proof starts only after the protocol contract and conformance entry rules are stable. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, adapters fourth, product proof last.</t>
+          <t>Near-term priority: make Jarvis OpenAPI-ready: protocol lock, OpenAPI 3.1 communication binding, version and capability negotiation, zero-trust security model, portable export, and conformance entry fixtures. Compatible example starts only after the protocol contract and conformance entry rules are stable. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, compatibility mapping fourth, compatible example last.</t>
         </is>
       </c>
       <c r="B4" s="30" t="n"/>
@@ -837,7 +837,7 @@
       <c r="F5" s="31" t="n"/>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>Proof Readiness</t>
+          <t>Compatibility Proof</t>
         </is>
       </c>
       <c r="H5" s="31" t="n"/>
@@ -870,12 +870,12 @@
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>Adapter + interoperability</t>
+          <t>Compatibility + interoperability</t>
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>Product proof</t>
+          <t>Compatible example</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
@@ -919,20 +919,20 @@
       </c>
       <c r="F7" s="21" t="inlineStr">
         <is>
-          <t>- defer adapter implementation
-- name adapter questions only
+          <t>- defer integration implementation
+- name compatibility questions only
 - preserve runtime independence</t>
         </is>
       </c>
       <c r="G7" s="22" t="inlineStr">
         <is>
-          <t>- keep Garden POC out of active scope
-- define product-proof prerequisites only</t>
+          <t>- keep host implementation work out of active scope
+- define compatible-example prerequisites only</t>
         </is>
       </c>
       <c r="H7" s="23" t="inlineStr">
         <is>
-          <t>Protocol lock is the source for OpenAPI work, OpenAPI 3.1 is the machine-readable communication contract, and no product proof enters this week.</t>
+          <t>Protocol lock is the source for OpenAPI work, OpenAPI 3.1 is the machine-readable communication contract, and no compatible example enters this week.</t>
         </is>
       </c>
     </row>
@@ -971,16 +971,16 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>- document adapter contract questions
-- define AgentWorker adapter surface
+          <t>- document compatibility mapping questions
+- define AgentWorker compatibility surface
 - define tool/action to PolicyDecision mapping
 - define limitations field for unsupported concepts</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>- keep Garden POC out of active scope
-- define product-proof gate conditions only</t>
+          <t>- keep host implementation work out of active scope
+- define compatible-example gate conditions only</t>
         </is>
       </c>
       <c r="H8" s="25" t="inlineStr">
@@ -1018,12 +1018,12 @@
           <t>- build golden-path fixtures
 - build failing fixtures
 - validate status transitions
-- validate export does not require product-private fields</t>
+- validate export does not require host-private fields</t>
         </is>
       </c>
       <c r="F9" s="21" t="inlineStr">
         <is>
-          <t>- create CLI/existing-agent adapter plan
+          <t>- create existing-agent compatibility plan
 - capture messages/actions as JarvisEvents
 - capture tool use as PolicyDecision and Evidence
 - capture human correction as Review</t>
@@ -1031,8 +1031,8 @@
       </c>
       <c r="G9" s="22" t="inlineStr">
         <is>
-          <t>- keep product proof out of active scope
-- record product-proof prerequisites from conformance only
+          <t>- keep compatible example out of active scope
+- record compatible-example prerequisites from conformance only
 - generate protocol-only sample WorkSession export
 - document host-only assumptions separately</t>
         </is>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>Prove Jarvis with conformance fixtures and one adapter contract.</t>
+          <t>Prove Jarvis with conformance fixtures and protocol compatibility mapping.</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr">
@@ -1070,14 +1070,14 @@
       <c r="E10" s="25" t="inlineStr">
         <is>
           <t>- run OpenAPI examples against host export
-- run OpenAPI examples against CLI/adapter export
+- run OpenAPI examples against second compatible export
 - compare both exports for same core semantics
 - record gaps as conformance issues</t>
         </is>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>- implement proof adapter path
+          <t>- define proof compatibility path
 - HumanWorker objective -&gt; AgentWorker action
 - blocked action -&gt; Request
 - human response -&gt; Review or Takeover</t>
@@ -1085,14 +1085,14 @@
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>- prepare Garden POC as later product proof
-- define product-private fields that stay out of export
+          <t>- prepare compatible examples after the conformance gate
+- define host-private fields that stay out of export
 - update simulation narrative if needed</t>
         </is>
       </c>
       <c r="H10" s="25" t="inlineStr">
         <is>
-          <t>Two different host or adapter shapes produce valid Jarvis records for the same collaboration loop without sharing runtime, UI, storage, or execution stack.</t>
+          <t>Two compatible implementation shapes produce valid Jarvis records for the same collaboration loop without sharing runtime, UI, storage, or execution stack.</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Freeze v0.1 alpha and prepare product-proof review.</t>
+          <t>Freeze v0.1 alpha and prepare compatible-example review.</t>
         </is>
       </c>
       <c r="D11" s="20" t="inlineStr">
@@ -1130,23 +1130,23 @@
       </c>
       <c r="F11" s="21" t="inlineStr">
         <is>
-          <t>- write adapter guide
-- document CLI/existing-agent adapter
-- document host implementation guide
-- identify next two adapter targets</t>
+          <t>- write compatibility mapping guide
+- document CLI/existing-agent compatibility mapping
+- document compatible implementation guide
+- identify next two compatibility targets</t>
         </is>
       </c>
       <c r="G11" s="22" t="inlineStr">
         <is>
           <t>- publish protocol proof walkthrough URL
-- package product-proof readiness notes
+- package compatible-example readiness notes
 - prepare team walkthrough
 - collect review notes into next-cycle issues</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr">
         <is>
-          <t>Jarvis has a v0.1 alpha package of protocol docs, OpenAPI contract, examples, conformance fixtures, product-proof readiness, and one existing-agent adapter contract.</t>
+          <t>Jarvis has a v0.1 alpha package of protocol docs, OpenAPI contract, examples, conformance fixtures, compatible-example readiness, and one existing-agent compatibility mapping.</t>
         </is>
       </c>
     </row>
@@ -1163,12 +1163,12 @@
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>Expand only from conformance results and product-proof evidence.</t>
+          <t>Expand only from conformance results and compatible-example evidence.</t>
         </is>
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>- harden object model from real adapters
+          <t>- harden object model from real compatible implementations
 - add migration rules
 - add public implementation checklist
 - prepare v0.2 evidence and learning beta</t>
@@ -1184,15 +1184,15 @@
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>- more agent adapters
+          <t>- more agent compatibility mappings
 - MCP/A2A/AG-UI integration notes
-- SDK-neutral adapter examples
+- SDK-neutral compatibility examples
 - compatibility badges</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>- additional product proofs
+          <t>- additional compatible examples
 - public proof refresh
 - team onboarding sheet
 - protocol review sessions</t>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="H12" s="25" t="inlineStr">
         <is>
-          <t>Expansion is justified by valid exports, conformance failures, adapter pain, and product-proof evidence, not by unproven feature expansion.</t>
+          <t>Expansion is justified by valid exports, conformance failures, compatibility pain, and compatible-example evidence, not by unproven feature expansion.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close Week 2 and set Week 3 focus (#28)
</commit_message>
<xml_diff>
--- a/docs/planning/sheets/jarvis_roadmap.xlsx
+++ b/docs/planning/sheets/jarvis_roadmap.xlsx
@@ -781,7 +781,7 @@
     <row r="2" ht="50" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Jarvis is the human-agent collaboration and learning-loop protocol. It defines WorkSession, Policy, Request, Review, Takeover, Contribution, EvidenceManifest, LearningRecord, MemoryProposal, and SkillProposal so existing agents and host products collaborate with humans without replacing their runtimes.</t>
+          <t>Jarvis is the human-agent collaboration and learning-loop protocol. It defines WorkSession, Policy, Request, Review, Takeover, Contribution, EvidenceManifest, LearningRecord, MemoryProposal, and SkillProposal so existing agents and host applications collaborate with humans without replacing their runtimes.</t>
         </is>
       </c>
       <c r="B2" s="32" t="n"/>
@@ -805,7 +805,7 @@
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Near-term priority: make Jarvis OpenAPI-ready: protocol lock, OpenAPI 3.1 communication binding, version and capability negotiation, zero-trust security model, portable export, and conformance entry fixtures. Product proof starts only after the protocol contract and conformance entry rules are stable. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, adapters fourth, product proof last.</t>
+          <t>Near-term priority: make Jarvis OpenAPI-ready: protocol lock, OpenAPI 3.1 communication binding, version and capability negotiation, zero-trust security model, portable export, and conformance entry fixtures. Compatible example starts only after the protocol contract and conformance entry rules are stable. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, compatibility mapping fourth, compatible example last.</t>
         </is>
       </c>
       <c r="B4" s="30" t="n"/>
@@ -837,7 +837,7 @@
       <c r="F5" s="31" t="n"/>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>Proof Readiness</t>
+          <t>Compatibility Proof</t>
         </is>
       </c>
       <c r="H5" s="31" t="n"/>
@@ -870,12 +870,12 @@
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>Adapter + interoperability</t>
+          <t>Compatibility + interoperability</t>
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>Product proof</t>
+          <t>Compatible example</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
@@ -919,20 +919,20 @@
       </c>
       <c r="F7" s="21" t="inlineStr">
         <is>
-          <t>- defer adapter implementation
-- name adapter questions only
+          <t>- defer integration implementation
+- name compatibility questions only
 - preserve runtime independence</t>
         </is>
       </c>
       <c r="G7" s="22" t="inlineStr">
         <is>
-          <t>- keep Garden POC out of active scope
-- define product-proof prerequisites only</t>
+          <t>- keep host implementation work out of active scope
+- define compatible-example prerequisites only</t>
         </is>
       </c>
       <c r="H7" s="23" t="inlineStr">
         <is>
-          <t>Protocol lock is the source for OpenAPI work, OpenAPI 3.1 is the machine-readable communication contract, and no product proof enters this week.</t>
+          <t>Protocol lock is the source for OpenAPI work, OpenAPI 3.1 is the machine-readable communication contract, and no compatible example enters this week.</t>
         </is>
       </c>
     </row>
@@ -971,16 +971,16 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>- document adapter contract questions
-- define AgentWorker adapter surface
+          <t>- document compatibility mapping questions
+- define AgentWorker compatibility surface
 - define tool/action to PolicyDecision mapping
 - define limitations field for unsupported concepts</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>- keep Garden POC out of active scope
-- define product-proof gate conditions only</t>
+          <t>- keep host implementation work out of active scope
+- define compatible-example gate conditions only</t>
         </is>
       </c>
       <c r="H8" s="25" t="inlineStr">
@@ -1018,12 +1018,12 @@
           <t>- build golden-path fixtures
 - build failing fixtures
 - validate status transitions
-- validate export does not require product-private fields</t>
+- validate export does not require host-private fields</t>
         </is>
       </c>
       <c r="F9" s="21" t="inlineStr">
         <is>
-          <t>- create CLI/existing-agent adapter plan
+          <t>- create existing-agent compatibility plan
 - capture messages/actions as JarvisEvents
 - capture tool use as PolicyDecision and Evidence
 - capture human correction as Review</t>
@@ -1031,8 +1031,8 @@
       </c>
       <c r="G9" s="22" t="inlineStr">
         <is>
-          <t>- keep product proof out of active scope
-- record product-proof prerequisites from conformance only
+          <t>- keep compatible example out of active scope
+- record compatible-example prerequisites from conformance only
 - generate protocol-only sample WorkSession export
 - document host-only assumptions separately</t>
         </is>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>Prove Jarvis with conformance fixtures and one adapter contract.</t>
+          <t>Prove Jarvis with conformance fixtures and protocol compatibility mapping.</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr">
@@ -1070,14 +1070,14 @@
       <c r="E10" s="25" t="inlineStr">
         <is>
           <t>- run OpenAPI examples against host export
-- run OpenAPI examples against CLI/adapter export
+- run OpenAPI examples against second compatible export
 - compare both exports for same core semantics
 - record gaps as conformance issues</t>
         </is>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>- implement proof adapter path
+          <t>- define proof compatibility path
 - HumanWorker objective -&gt; AgentWorker action
 - blocked action -&gt; Request
 - human response -&gt; Review or Takeover</t>
@@ -1085,14 +1085,14 @@
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>- prepare Garden POC as later product proof
-- define product-private fields that stay out of export
+          <t>- prepare compatible examples after the conformance gate
+- define host-private fields that stay out of export
 - update simulation narrative if needed</t>
         </is>
       </c>
       <c r="H10" s="25" t="inlineStr">
         <is>
-          <t>Two different host or adapter shapes produce valid Jarvis records for the same collaboration loop without sharing runtime, UI, storage, or execution stack.</t>
+          <t>Two compatible implementation shapes produce valid Jarvis records for the same collaboration loop without sharing runtime, UI, storage, or execution stack.</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Freeze v0.1 alpha and prepare product-proof review.</t>
+          <t>Freeze v0.1 alpha and prepare compatible-example review.</t>
         </is>
       </c>
       <c r="D11" s="20" t="inlineStr">
@@ -1130,23 +1130,23 @@
       </c>
       <c r="F11" s="21" t="inlineStr">
         <is>
-          <t>- write adapter guide
-- document CLI/existing-agent adapter
-- document host implementation guide
-- identify next two adapter targets</t>
+          <t>- write compatibility mapping guide
+- document CLI/existing-agent compatibility mapping
+- document compatible implementation guide
+- identify next two compatibility targets</t>
         </is>
       </c>
       <c r="G11" s="22" t="inlineStr">
         <is>
           <t>- publish protocol proof walkthrough URL
-- package product-proof readiness notes
+- package compatible-example readiness notes
 - prepare team walkthrough
 - collect review notes into next-cycle issues</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr">
         <is>
-          <t>Jarvis has a v0.1 alpha package of protocol docs, OpenAPI contract, examples, conformance fixtures, product-proof readiness, and one existing-agent adapter contract.</t>
+          <t>Jarvis has a v0.1 alpha package of protocol docs, OpenAPI contract, examples, conformance fixtures, compatible-example readiness, and one existing-agent compatibility mapping.</t>
         </is>
       </c>
     </row>
@@ -1163,12 +1163,12 @@
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>Expand only from conformance results and product-proof evidence.</t>
+          <t>Expand only from conformance results and compatible-example evidence.</t>
         </is>
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>- harden object model from real adapters
+          <t>- harden object model from real compatible implementations
 - add migration rules
 - add public implementation checklist
 - prepare v0.2 evidence and learning beta</t>
@@ -1184,15 +1184,15 @@
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>- more agent adapters
+          <t>- more agent compatibility mappings
 - MCP/A2A/AG-UI integration notes
-- SDK-neutral adapter examples
+- SDK-neutral compatibility examples
 - compatibility badges</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>- additional product proofs
+          <t>- additional compatible examples
 - public proof refresh
 - team onboarding sheet
 - protocol review sessions</t>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="H12" s="25" t="inlineStr">
         <is>
-          <t>Expansion is justified by valid exports, conformance failures, adapter pain, and product-proof evidence, not by unproven feature expansion.</t>
+          <t>Expansion is justified by valid exports, conformance failures, compatibility pain, and compatible-example evidence, not by unproven feature expansion.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tighten v0.1 pre-tag audit contract
</commit_message>
<xml_diff>
--- a/docs/planning/sheets/jarvis_roadmap.xlsx
+++ b/docs/planning/sheets/jarvis_roadmap.xlsx
@@ -805,7 +805,7 @@
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Near-term priority: make Jarvis OpenAPI-ready: protocol lock, OpenAPI 3.1 communication binding, version and capability negotiation, zero-trust security model, portable export, and conformance entry fixtures. Compatible example starts only after the protocol contract and conformance entry rules are stable. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, compatibility mapping fourth, compatible example last.</t>
+          <t>Near-term priority: maintain the v0.1.0 Protocol Alpha contract and define next-phase protocol targets after acceptance review. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, compatibility mapping fourth, compatible example last.</t>
         </is>
       </c>
       <c r="B4" s="30" t="n"/>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Freeze v0.1 alpha and prepare compatible-example review.</t>
+          <t>Close v0.1.0 Protocol Alpha and prepare compatible-example review.</t>
         </is>
       </c>
       <c r="D11" s="20" t="inlineStr">
@@ -1187,7 +1187,8 @@
           <t>- more agent compatibility mappings
 - MCP/A2A/AG-UI integration notes
 - SDK-neutral compatibility examples
-- compatibility badges</t>
+- compatibility evidence labels and claim-format examples
+- no certification or adopter badge</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">

</xml_diff>

<commit_message>
[codex] Tighten v0.1 public readiness docs (#58)
* Clarify v0.1 acceptance release status

* Tighten v0.1 public readiness docs

* Remove stale release preparation wording

* Tighten v0.1 pre-tag audit contract

* Complete final v0.1 pre-tag audit
</commit_message>
<xml_diff>
--- a/docs/planning/sheets/jarvis_roadmap.xlsx
+++ b/docs/planning/sheets/jarvis_roadmap.xlsx
@@ -805,7 +805,7 @@
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Near-term priority: make Jarvis OpenAPI-ready: protocol lock, OpenAPI 3.1 communication binding, version and capability negotiation, zero-trust security model, portable export, and conformance entry fixtures. Compatible example starts only after the protocol contract and conformance entry rules are stable. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, compatibility mapping fourth, compatible example last.</t>
+          <t>Near-term priority: maintain the v0.1.0 Protocol Alpha contract and define next-phase protocol targets after acceptance review. Keep scope narrow: protocol records first, OpenAPI contract second, conformance third, compatibility mapping fourth, compatible example last.</t>
         </is>
       </c>
       <c r="B4" s="30" t="n"/>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Freeze v0.1 alpha and prepare compatible-example review.</t>
+          <t>Close v0.1.0 Protocol Alpha and prepare compatible-example review.</t>
         </is>
       </c>
       <c r="D11" s="20" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="H11" s="23" t="inlineStr">
         <is>
-          <t>Jarvis has a v0.1 alpha package of protocol docs, OpenAPI contract, examples, conformance fixtures, compatible-example readiness, and one existing-agent compatibility mapping.</t>
+          <t>Jarvis has a v0.1.0 Protocol Alpha package of protocol docs, OpenAPI contract, examples, conformance fixtures, compatible-example readiness, and one existing-agent compatibility mapping.</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1187,8 @@
           <t>- more agent compatibility mappings
 - MCP/A2A/AG-UI integration notes
 - SDK-neutral compatibility examples
-- compatibility badges</t>
+- compatibility evidence labels and claim-format examples
+- no certification or adopter badge</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">

</xml_diff>